<commit_message>
dev: more rebase notes
</commit_message>
<xml_diff>
--- a/~devEnv/rebase-commits.xlsx
+++ b/~devEnv/rebase-commits.xlsx
@@ -8,24 +8,29 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DSPEER\AppData\Roaming\FreeCAD\v1-1\Mod\CurvedShapesWorkbench\~devEnv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{629EB8A0-285E-4280-A96F-A36AA1BCBCC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3518B1A2-0AE1-40D5-9EDF-10C0557619CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{65AC9CD5-7DF8-4DF6-8DC5-A63C69A8CCB7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{65AC9CD5-7DF8-4DF6-8DC5-A63C69A8CCB7}"/>
   </bookViews>
   <sheets>
     <sheet name="rebase-commits orig" sheetId="1" r:id="rId1"/>
     <sheet name="mod pivot files" sheetId="3" r:id="rId2"/>
-    <sheet name="rebase-commits mod" sheetId="2" r:id="rId3"/>
+    <sheet name="manual file identification" sheetId="4" r:id="rId3"/>
+    <sheet name="rebase-commits mod" sheetId="2" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'manual file identification'!$A$1:$B$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'rebase-commits mod'!$A$1:$F$144</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
   <pivotCaches>
-    <pivotCache cacheId="3" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId5"/>
   </pivotCaches>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1235" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1389" uniqueCount="211">
   <si>
     <t>sha</t>
   </si>
@@ -649,6 +654,15 @@
   </si>
   <si>
     <t>Count of sha</t>
+  </si>
+  <si>
+    <t>feature pr</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>yes</t>
   </si>
 </sst>
 </file>
@@ -1132,14 +1146,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2467,7 +2480,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FA9F2681-C01C-47D6-AF1C-88971D39D327}" name="PivotTable1" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FA9F2681-C01C-47D6-AF1C-88971D39D327}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B81" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="6">
     <pivotField showAll="0"/>
@@ -5616,7 +5629,7 @@
       <c r="A4" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4">
         <v>1</v>
       </c>
     </row>
@@ -5624,7 +5637,7 @@
       <c r="A5" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5">
         <v>1</v>
       </c>
     </row>
@@ -5632,7 +5645,7 @@
       <c r="A6" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6">
         <v>1</v>
       </c>
     </row>
@@ -5640,7 +5653,7 @@
       <c r="A7" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7">
         <v>1</v>
       </c>
     </row>
@@ -5648,7 +5661,7 @@
       <c r="A8" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8">
         <v>1</v>
       </c>
     </row>
@@ -5656,7 +5669,7 @@
       <c r="A9" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9">
         <v>3</v>
       </c>
     </row>
@@ -5664,7 +5677,7 @@
       <c r="A10" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B10" s="4">
+      <c r="B10">
         <v>1</v>
       </c>
     </row>
@@ -5672,7 +5685,7 @@
       <c r="A11" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="4">
+      <c r="B11">
         <v>1</v>
       </c>
     </row>
@@ -5680,7 +5693,7 @@
       <c r="A12" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B12" s="4">
+      <c r="B12">
         <v>1</v>
       </c>
     </row>
@@ -5688,7 +5701,7 @@
       <c r="A13" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="4">
+      <c r="B13">
         <v>1</v>
       </c>
     </row>
@@ -5696,7 +5709,7 @@
       <c r="A14" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="4">
+      <c r="B14">
         <v>1</v>
       </c>
     </row>
@@ -5704,7 +5717,7 @@
       <c r="A15" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="4">
+      <c r="B15">
         <v>1</v>
       </c>
     </row>
@@ -5712,7 +5725,7 @@
       <c r="A16" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B16" s="4">
+      <c r="B16">
         <v>1</v>
       </c>
     </row>
@@ -5720,7 +5733,7 @@
       <c r="A17" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B17" s="4">
+      <c r="B17">
         <v>1</v>
       </c>
     </row>
@@ -5728,7 +5741,7 @@
       <c r="A18" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B18" s="4">
+      <c r="B18">
         <v>1</v>
       </c>
     </row>
@@ -5736,7 +5749,7 @@
       <c r="A19" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B19" s="4">
+      <c r="B19">
         <v>1</v>
       </c>
     </row>
@@ -5744,7 +5757,7 @@
       <c r="A20" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B20" s="4">
+      <c r="B20">
         <v>1</v>
       </c>
     </row>
@@ -5752,7 +5765,7 @@
       <c r="A21" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B21" s="4">
+      <c r="B21">
         <v>1</v>
       </c>
     </row>
@@ -5760,7 +5773,7 @@
       <c r="A22" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B22" s="4">
+      <c r="B22">
         <v>1</v>
       </c>
     </row>
@@ -5768,7 +5781,7 @@
       <c r="A23" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B23" s="4">
+      <c r="B23">
         <v>1</v>
       </c>
     </row>
@@ -5776,7 +5789,7 @@
       <c r="A24" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B24" s="4">
+      <c r="B24">
         <v>1</v>
       </c>
     </row>
@@ -5784,7 +5797,7 @@
       <c r="A25" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B25" s="4">
+      <c r="B25">
         <v>1</v>
       </c>
     </row>
@@ -5792,7 +5805,7 @@
       <c r="A26" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B26" s="4">
+      <c r="B26">
         <v>1</v>
       </c>
     </row>
@@ -5800,7 +5813,7 @@
       <c r="A27" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B27" s="4">
+      <c r="B27">
         <v>1</v>
       </c>
     </row>
@@ -5808,7 +5821,7 @@
       <c r="A28" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B28" s="4">
+      <c r="B28">
         <v>1</v>
       </c>
     </row>
@@ -5816,7 +5829,7 @@
       <c r="A29" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B29" s="4">
+      <c r="B29">
         <v>2</v>
       </c>
     </row>
@@ -5824,7 +5837,7 @@
       <c r="A30" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="B30" s="4">
+      <c r="B30">
         <v>1</v>
       </c>
     </row>
@@ -5832,7 +5845,7 @@
       <c r="A31" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="4">
+      <c r="B31">
         <v>6</v>
       </c>
     </row>
@@ -5840,7 +5853,7 @@
       <c r="A32" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="B32" s="4">
+      <c r="B32">
         <v>1</v>
       </c>
     </row>
@@ -5848,7 +5861,7 @@
       <c r="A33" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B33" s="4">
+      <c r="B33">
         <v>2</v>
       </c>
     </row>
@@ -5856,7 +5869,7 @@
       <c r="A34" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B34" s="4">
+      <c r="B34">
         <v>2</v>
       </c>
     </row>
@@ -5864,7 +5877,7 @@
       <c r="A35" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B35" s="4">
+      <c r="B35">
         <v>2</v>
       </c>
     </row>
@@ -5872,7 +5885,7 @@
       <c r="A36" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B36" s="4">
+      <c r="B36">
         <v>2</v>
       </c>
     </row>
@@ -5880,7 +5893,7 @@
       <c r="A37" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B37" s="4">
+      <c r="B37">
         <v>2</v>
       </c>
     </row>
@@ -5888,7 +5901,7 @@
       <c r="A38" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B38" s="4">
+      <c r="B38">
         <v>2</v>
       </c>
     </row>
@@ -5896,7 +5909,7 @@
       <c r="A39" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B39" s="4">
+      <c r="B39">
         <v>3</v>
       </c>
     </row>
@@ -5904,7 +5917,7 @@
       <c r="A40" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B40" s="4">
+      <c r="B40">
         <v>2</v>
       </c>
     </row>
@@ -5912,7 +5925,7 @@
       <c r="A41" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="B41" s="4">
+      <c r="B41">
         <v>1</v>
       </c>
     </row>
@@ -5920,7 +5933,7 @@
       <c r="A42" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="B42" s="4">
+      <c r="B42">
         <v>1</v>
       </c>
     </row>
@@ -5928,7 +5941,7 @@
       <c r="A43" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="B43" s="4">
+      <c r="B43">
         <v>1</v>
       </c>
     </row>
@@ -5936,7 +5949,7 @@
       <c r="A44" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="B44" s="4">
+      <c r="B44">
         <v>1</v>
       </c>
     </row>
@@ -5944,7 +5957,7 @@
       <c r="A45" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="B45" s="4">
+      <c r="B45">
         <v>1</v>
       </c>
     </row>
@@ -5952,7 +5965,7 @@
       <c r="A46" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="B46" s="4">
+      <c r="B46">
         <v>1</v>
       </c>
     </row>
@@ -5960,7 +5973,7 @@
       <c r="A47" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="B47" s="4">
+      <c r="B47">
         <v>3</v>
       </c>
     </row>
@@ -5968,7 +5981,7 @@
       <c r="A48" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="B48" s="4">
+      <c r="B48">
         <v>1</v>
       </c>
     </row>
@@ -5976,7 +5989,7 @@
       <c r="A49" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B49" s="4">
+      <c r="B49">
         <v>2</v>
       </c>
     </row>
@@ -5984,7 +5997,7 @@
       <c r="A50" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="B50" s="4">
+      <c r="B50">
         <v>1</v>
       </c>
     </row>
@@ -5992,7 +6005,7 @@
       <c r="A51" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B51" s="4">
+      <c r="B51">
         <v>6</v>
       </c>
     </row>
@@ -6000,7 +6013,7 @@
       <c r="A52" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="B52" s="4">
+      <c r="B52">
         <v>1</v>
       </c>
     </row>
@@ -6008,7 +6021,7 @@
       <c r="A53" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="B53" s="4">
+      <c r="B53">
         <v>1</v>
       </c>
     </row>
@@ -6016,7 +6029,7 @@
       <c r="A54" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="B54" s="4">
+      <c r="B54">
         <v>1</v>
       </c>
     </row>
@@ -6024,7 +6037,7 @@
       <c r="A55" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="B55" s="4">
+      <c r="B55">
         <v>1</v>
       </c>
     </row>
@@ -6032,7 +6045,7 @@
       <c r="A56" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="B56" s="4">
+      <c r="B56">
         <v>1</v>
       </c>
     </row>
@@ -6040,7 +6053,7 @@
       <c r="A57" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="B57" s="4">
+      <c r="B57">
         <v>1</v>
       </c>
     </row>
@@ -6048,7 +6061,7 @@
       <c r="A58" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="B58" s="4">
+      <c r="B58">
         <v>1</v>
       </c>
     </row>
@@ -6056,7 +6069,7 @@
       <c r="A59" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="B59" s="4">
+      <c r="B59">
         <v>2</v>
       </c>
     </row>
@@ -6064,7 +6077,7 @@
       <c r="A60" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="B60" s="4">
+      <c r="B60">
         <v>2</v>
       </c>
     </row>
@@ -6072,7 +6085,7 @@
       <c r="A61" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="B61" s="4">
+      <c r="B61">
         <v>1</v>
       </c>
     </row>
@@ -6080,7 +6093,7 @@
       <c r="A62" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="B62" s="4">
+      <c r="B62">
         <v>2</v>
       </c>
     </row>
@@ -6088,7 +6101,7 @@
       <c r="A63" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="B63" s="4">
+      <c r="B63">
         <v>2</v>
       </c>
     </row>
@@ -6096,7 +6109,7 @@
       <c r="A64" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="B64" s="4">
+      <c r="B64">
         <v>1</v>
       </c>
     </row>
@@ -6104,7 +6117,7 @@
       <c r="A65" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="B65" s="4">
+      <c r="B65">
         <v>1</v>
       </c>
     </row>
@@ -6112,7 +6125,7 @@
       <c r="A66" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="B66" s="4">
+      <c r="B66">
         <v>1</v>
       </c>
     </row>
@@ -6120,7 +6133,7 @@
       <c r="A67" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="B67" s="4">
+      <c r="B67">
         <v>2</v>
       </c>
     </row>
@@ -6128,7 +6141,7 @@
       <c r="A68" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="B68" s="4">
+      <c r="B68">
         <v>1</v>
       </c>
     </row>
@@ -6136,7 +6149,7 @@
       <c r="A69" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="B69" s="4">
+      <c r="B69">
         <v>5</v>
       </c>
     </row>
@@ -6144,7 +6157,7 @@
       <c r="A70" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="B70" s="4">
+      <c r="B70">
         <v>1</v>
       </c>
     </row>
@@ -6152,7 +6165,7 @@
       <c r="A71" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="B71" s="4">
+      <c r="B71">
         <v>2</v>
       </c>
     </row>
@@ -6160,7 +6173,7 @@
       <c r="A72" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="B72" s="4">
+      <c r="B72">
         <v>2</v>
       </c>
     </row>
@@ -6168,7 +6181,7 @@
       <c r="A73" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="B73" s="4">
+      <c r="B73">
         <v>2</v>
       </c>
     </row>
@@ -6176,7 +6189,7 @@
       <c r="A74" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B74" s="4">
+      <c r="B74">
         <v>22</v>
       </c>
     </row>
@@ -6184,7 +6197,7 @@
       <c r="A75" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="B75" s="4">
+      <c r="B75">
         <v>2</v>
       </c>
     </row>
@@ -6192,7 +6205,7 @@
       <c r="A76" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="B76" s="4">
+      <c r="B76">
         <v>1</v>
       </c>
     </row>
@@ -6200,7 +6213,7 @@
       <c r="A77" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B77" s="4">
+      <c r="B77">
         <v>8</v>
       </c>
     </row>
@@ -6208,7 +6221,7 @@
       <c r="A78" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B78" s="4">
+      <c r="B78">
         <v>1</v>
       </c>
     </row>
@@ -6216,7 +6229,7 @@
       <c r="A79" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="B79" s="4">
+      <c r="B79">
         <v>2</v>
       </c>
     </row>
@@ -6224,13 +6237,12 @@
       <c r="A80" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="B80" s="4"/>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="B81" s="4">
+      <c r="B81">
         <v>143</v>
       </c>
     </row>
@@ -6240,7 +6252,646 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66A4BAB0-06B4-4A76-B404-BDC160FF826D}">
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:B77"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="70.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>181</v>
+      </c>
+      <c r="B2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>202</v>
+      </c>
+      <c r="B3" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>190</v>
+      </c>
+      <c r="B5" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>189</v>
+      </c>
+      <c r="B6" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>137</v>
+      </c>
+      <c r="B7" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>64</v>
+      </c>
+      <c r="B14" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>71</v>
+      </c>
+      <c r="B15" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>65</v>
+      </c>
+      <c r="B16" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>66</v>
+      </c>
+      <c r="B17" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>67</v>
+      </c>
+      <c r="B18" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>68</v>
+      </c>
+      <c r="B19" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>69</v>
+      </c>
+      <c r="B20" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>70</v>
+      </c>
+      <c r="B21" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>51</v>
+      </c>
+      <c r="B22" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>38</v>
+      </c>
+      <c r="B23" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>33</v>
+      </c>
+      <c r="B24" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>21</v>
+      </c>
+      <c r="B26" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>14</v>
+      </c>
+      <c r="B27" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>72</v>
+      </c>
+      <c r="B28" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>15</v>
+      </c>
+      <c r="B29" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>109</v>
+      </c>
+      <c r="B30" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>56</v>
+      </c>
+      <c r="B31" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>63</v>
+      </c>
+      <c r="B32" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>57</v>
+      </c>
+      <c r="B33" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>58</v>
+      </c>
+      <c r="B34" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>59</v>
+      </c>
+      <c r="B35" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>60</v>
+      </c>
+      <c r="B36" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>61</v>
+      </c>
+      <c r="B37" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>143</v>
+      </c>
+      <c r="B39" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>144</v>
+      </c>
+      <c r="B40" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>145</v>
+      </c>
+      <c r="B41" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>106</v>
+      </c>
+      <c r="B42" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>146</v>
+      </c>
+      <c r="B43" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>147</v>
+      </c>
+      <c r="B44" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>73</v>
+      </c>
+      <c r="B45" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>155</v>
+      </c>
+      <c r="B46" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>74</v>
+      </c>
+      <c r="B47" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>191</v>
+      </c>
+      <c r="B48" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>52</v>
+      </c>
+      <c r="B49" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>192</v>
+      </c>
+      <c r="B50" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>193</v>
+      </c>
+      <c r="B51" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>194</v>
+      </c>
+      <c r="B52" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>195</v>
+      </c>
+      <c r="B53" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>196</v>
+      </c>
+      <c r="B54" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>197</v>
+      </c>
+      <c r="B55" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>198</v>
+      </c>
+      <c r="B56" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>158</v>
+      </c>
+      <c r="B57" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>159</v>
+      </c>
+      <c r="B58" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>162</v>
+      </c>
+      <c r="B59" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>163</v>
+      </c>
+      <c r="B60" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>164</v>
+      </c>
+      <c r="B61" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>130</v>
+      </c>
+      <c r="B62" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>115</v>
+      </c>
+      <c r="B63" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>148</v>
+      </c>
+      <c r="B64" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>114</v>
+      </c>
+      <c r="B65" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>199</v>
+      </c>
+      <c r="B66" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>97</v>
+      </c>
+      <c r="B67" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>178</v>
+      </c>
+      <c r="B68" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>186</v>
+      </c>
+      <c r="B69" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>185</v>
+      </c>
+      <c r="B70" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>184</v>
+      </c>
+      <c r="B71" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>8</v>
+      </c>
+      <c r="B72" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>187</v>
+      </c>
+      <c r="B73" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>140</v>
+      </c>
+      <c r="B74" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>9</v>
+      </c>
+      <c r="B75" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>11</v>
+      </c>
+      <c r="B76" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>188</v>
+      </c>
+      <c r="B77" t="s">
+        <v>209</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B77" xr:uid="{66A4BAB0-06B4-4A76-B404-BDC160FF826D}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="no"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3784EE7-2821-4222-900C-20895030BFEF}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:F144"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -6371,7 +7022,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -6391,7 +7042,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -6411,7 +7062,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -6471,7 +7122,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -6491,7 +7142,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -6511,7 +7162,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -6571,7 +7222,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -6591,7 +7242,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -6611,7 +7262,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -6671,7 +7322,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -6691,7 +7342,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -6711,7 +7362,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -6771,7 +7422,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -6791,7 +7442,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -6811,7 +7462,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -6831,7 +7482,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -6891,7 +7542,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -6931,7 +7582,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -6951,7 +7602,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -6991,7 +7642,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -7011,7 +7662,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -7031,7 +7682,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -7051,7 +7702,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -7071,7 +7722,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -7091,7 +7742,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -7111,7 +7762,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -7131,7 +7782,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -7151,7 +7802,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -7171,7 +7822,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -7191,7 +7842,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -7211,7 +7862,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
@@ -7231,7 +7882,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
@@ -7251,7 +7902,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
@@ -7271,7 +7922,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
@@ -7291,7 +7942,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
@@ -7311,7 +7962,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
@@ -7331,7 +7982,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>54</v>
       </c>
@@ -7351,7 +8002,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
@@ -7371,7 +8022,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>56</v>
       </c>
@@ -7391,7 +8042,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
@@ -7451,7 +8102,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
@@ -7471,7 +8122,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
@@ -7491,7 +8142,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>62</v>
       </c>
@@ -7511,7 +8162,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>63</v>
       </c>
@@ -7531,7 +8182,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>64</v>
       </c>
@@ -7551,7 +8202,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>65</v>
       </c>
@@ -7571,7 +8222,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>66</v>
       </c>
@@ -7591,7 +8242,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>67</v>
       </c>
@@ -7611,7 +8262,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>68</v>
       </c>
@@ -7631,7 +8282,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>69</v>
       </c>
@@ -7651,7 +8302,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>70</v>
       </c>
@@ -7671,7 +8322,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>71</v>
       </c>
@@ -7771,7 +8422,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>76</v>
       </c>
@@ -7791,7 +8442,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>77</v>
       </c>
@@ -7811,7 +8462,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>78</v>
       </c>
@@ -7831,7 +8482,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>79</v>
       </c>
@@ -7851,7 +8502,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>80</v>
       </c>
@@ -7991,7 +8642,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>87</v>
       </c>
@@ -8051,7 +8702,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>90</v>
       </c>
@@ -8071,7 +8722,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>91</v>
       </c>
@@ -8131,7 +8782,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>94</v>
       </c>
@@ -8151,7 +8802,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>95</v>
       </c>
@@ -8171,7 +8822,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>96</v>
       </c>
@@ -8191,7 +8842,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>97</v>
       </c>
@@ -8211,7 +8862,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>98</v>
       </c>
@@ -8231,7 +8882,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>99</v>
       </c>
@@ -8251,7 +8902,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>100</v>
       </c>
@@ -8271,7 +8922,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>101</v>
       </c>
@@ -8291,7 +8942,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>102</v>
       </c>
@@ -8311,7 +8962,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>103</v>
       </c>
@@ -8331,7 +8982,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>104</v>
       </c>
@@ -8351,7 +9002,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>105</v>
       </c>
@@ -8371,7 +9022,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>106</v>
       </c>
@@ -8391,7 +9042,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>107</v>
       </c>
@@ -8411,7 +9062,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>108</v>
       </c>
@@ -8431,7 +9082,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>109</v>
       </c>
@@ -8451,7 +9102,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>110</v>
       </c>
@@ -8491,7 +9142,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>112</v>
       </c>
@@ -8531,7 +9182,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>114</v>
       </c>
@@ -8551,7 +9202,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>115</v>
       </c>
@@ -8611,7 +9262,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>118</v>
       </c>
@@ -8631,7 +9282,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>119</v>
       </c>
@@ -8651,7 +9302,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>120</v>
       </c>
@@ -8671,7 +9322,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>121</v>
       </c>
@@ -8691,7 +9342,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>122</v>
       </c>
@@ -8711,7 +9362,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>123</v>
       </c>
@@ -8731,7 +9382,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>124</v>
       </c>
@@ -8751,7 +9402,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>125</v>
       </c>
@@ -8771,7 +9422,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>126</v>
       </c>
@@ -8791,7 +9442,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>127</v>
       </c>
@@ -8811,7 +9462,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>128</v>
       </c>
@@ -8831,7 +9482,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>129</v>
       </c>
@@ -8851,7 +9502,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>130</v>
       </c>
@@ -8871,7 +9522,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>131</v>
       </c>
@@ -8891,7 +9542,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>132</v>
       </c>
@@ -8911,7 +9562,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>133</v>
       </c>
@@ -8931,7 +9582,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>134</v>
       </c>
@@ -8951,7 +9602,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>135</v>
       </c>
@@ -8971,7 +9622,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>136</v>
       </c>
@@ -8991,7 +9642,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>137</v>
       </c>
@@ -9031,7 +9682,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>139</v>
       </c>
@@ -9051,7 +9702,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>140</v>
       </c>
@@ -9071,7 +9722,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>141</v>
       </c>
@@ -9091,7 +9742,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>142</v>
       </c>
@@ -9111,7 +9762,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>143</v>
       </c>
@@ -9132,6 +9783,18 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F144" xr:uid="{F3784EE7-2821-4222-900C-20895030BFEF}">
+    <filterColumn colId="5">
+      <filters>
+        <filter val="./CurvedArray.py"/>
+        <filter val="./CurvedShapes.py"/>
+        <filter val="./FishingLure.py"/>
+        <filter val="./InitGui.py"/>
+        <filter val="./README.md"/>
+        <filter val="./Resources/icons/FishingLure.svg"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>